<commit_message>
강남, 신촌 report, ppt 수정
</commit_message>
<xml_diff>
--- a/연구코드/aec/results/강남/feature_selection_report.xlsx
+++ b/연구코드/aec/results/강남/feature_selection_report.xlsx
@@ -11,9 +11,10 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="상관계수_Top20" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="VIF_선택feature" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="VIF_부분제거_비교" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TAMA_분포_성별" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CT_스캐너_분포" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="kVp_분포" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Correlation_Matrix" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TAMA_분포_성별" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CT_스캐너_분포" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="kVp_분포" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -3603,7 +3604,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C8"/>
+  <dimension ref="A1:C7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3626,11 +3627,11 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>p25</t>
+          <t>CV</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>72.17700000000001</v>
+        <v>1.579</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -3645,7 +3646,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>58.252</v>
+        <v>1.528</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -3656,11 +3657,11 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>CV</t>
+          <t>skewness</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>3.567</v>
+        <v>1.49</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -3671,11 +3672,11 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>skewness</t>
+          <t>slope_abs_mean</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>2.351</v>
+        <v>1.418</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -3686,11 +3687,11 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>slope_abs_mean</t>
+          <t>Sex</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>1.445</v>
+        <v>1.26</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -3701,28 +3702,13 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Sex</t>
+          <t>PatientAge</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>1.268</v>
+        <v>1.147</v>
       </c>
       <c r="C7" t="inlineStr">
-        <is>
-          <t>현재 선택 (SELECTED_AEC_FEATURES)</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>PatientAge</t>
-        </is>
-      </c>
-      <c r="B8" t="n">
-        <v>1.149</v>
-      </c>
-      <c r="C8" t="inlineStr">
         <is>
           <t>현재 선택 (SELECTED_AEC_FEATURES)</t>
         </is>
@@ -3739,7 +3725,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C31"/>
+  <dimension ref="A1:C27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3762,11 +3748,11 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>p25</t>
+          <t>CV</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>72.17700000000001</v>
+        <v>1.579</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -3781,7 +3767,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>58.252</v>
+        <v>1.528</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -3792,11 +3778,11 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>CV</t>
+          <t>skewness</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>3.567</v>
+        <v>1.49</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -3807,11 +3793,11 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>skewness</t>
+          <t>slope_abs_mean</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>2.351</v>
+        <v>1.418</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -3822,11 +3808,11 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>slope_abs_mean</t>
+          <t>Sex</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>1.445</v>
+        <v>1.26</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -3837,11 +3823,11 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Sex</t>
+          <t>PatientAge</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>1.268</v>
+        <v>1.147</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -3852,26 +3838,26 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>PatientAge</t>
+          <t>CV</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>1.149</v>
+        <v>1.578</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>현재 선택 (SELECTED_AEC_FEATURES)</t>
+          <t>mean 제외, AUC_normalized 포함</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>p25</t>
+          <t>AUC_normalized</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>71.973</v>
+        <v>1.527</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
@@ -3882,11 +3868,11 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>AUC_normalized</t>
+          <t>skewness</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>58.02</v>
+        <v>1.491</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
@@ -3897,11 +3883,11 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>CV</t>
+          <t>slope_abs_mean</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>3.59</v>
+        <v>1.415</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
@@ -3912,11 +3898,11 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>skewness</t>
+          <t>Sex</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>2.334</v>
+        <v>1.26</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
@@ -3927,11 +3913,11 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>slope_abs_mean</t>
+          <t>PatientAge</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>1.438</v>
+        <v>1.147</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
@@ -3942,43 +3928,45 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Sex</t>
-        </is>
-      </c>
-      <c r="B14" t="n">
-        <v>1.267</v>
+          <t>mean</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>inf</t>
+        </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>mean 제외, AUC_normalized 포함</t>
+          <t>AUC_normalized 제외, mean 포함</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>PatientAge</t>
-        </is>
-      </c>
-      <c r="B15" t="n">
-        <v>1.148</v>
+          <t>CV</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>inf</t>
+        </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>mean 제외, AUC_normalized 포함</t>
+          <t>AUC_normalized 제외, mean 포함</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>mean</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>inf</t>
-        </is>
+          <t>skewness</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>1.579</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
@@ -3989,13 +3977,11 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>mean</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>inf</t>
-        </is>
+          <t>slope_abs_mean</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>1.49</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
@@ -4006,11 +3992,11 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>p25</t>
+          <t>mean</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>72.17700000000001</v>
+        <v>1.418</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
@@ -4021,11 +4007,11 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>CV</t>
+          <t>Sex</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>3.567</v>
+        <v>1.26</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
@@ -4036,11 +4022,11 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>skewness</t>
+          <t>PatientAge</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>2.351</v>
+        <v>1.147</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
@@ -4051,56 +4037,56 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>slope_abs_mean</t>
+          <t>mean</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>1.445</v>
+        <v>57093.496</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>AUC_normalized 제외, mean 포함</t>
+          <t>mean + AUC_normalized 둘 다 포함</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Sex</t>
+          <t>AUC_normalized</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>1.268</v>
+        <v>57027.161</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>AUC_normalized 제외, mean 포함</t>
+          <t>mean + AUC_normalized 둘 다 포함</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>PatientAge</t>
+          <t>CV</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>1.149</v>
+        <v>1.69</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>AUC_normalized 제외, mean 포함</t>
+          <t>mean + AUC_normalized 둘 다 포함</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>mean</t>
+          <t>slope_abs_mean</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>57304.896</v>
+        <v>1.606</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
@@ -4111,11 +4097,11 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>AUC_normalized</t>
+          <t>skewness</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>57076.173</v>
+        <v>1.563</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
@@ -4126,11 +4112,11 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>p25</t>
+          <t>Sex</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>72.239</v>
+        <v>1.3</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
@@ -4141,73 +4127,13 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>CV</t>
+          <t>PatientAge</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>3.652</v>
+        <v>1.173</v>
       </c>
       <c r="C27" t="inlineStr">
-        <is>
-          <t>mean + AUC_normalized 둘 다 포함</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>skewness</t>
-        </is>
-      </c>
-      <c r="B28" t="n">
-        <v>2.439</v>
-      </c>
-      <c r="C28" t="inlineStr">
-        <is>
-          <t>mean + AUC_normalized 둘 다 포함</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>slope_abs_mean</t>
-        </is>
-      </c>
-      <c r="B29" t="n">
-        <v>1.638</v>
-      </c>
-      <c r="C29" t="inlineStr">
-        <is>
-          <t>mean + AUC_normalized 둘 다 포함</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>Sex</t>
-        </is>
-      </c>
-      <c r="B30" t="n">
-        <v>1.309</v>
-      </c>
-      <c r="C30" t="inlineStr">
-        <is>
-          <t>mean + AUC_normalized 둘 다 포함</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>PatientAge</t>
-        </is>
-      </c>
-      <c r="B31" t="n">
-        <v>1.176</v>
-      </c>
-      <c r="C31" t="inlineStr">
         <is>
           <t>mean + AUC_normalized 둘 다 포함</t>
         </is>
@@ -4224,138 +4150,189 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K3"/>
+  <dimension ref="A1:G7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>PatientAge</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Sex</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Mean</t>
-        </is>
-      </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>SD</t>
+          <t>mean</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Min</t>
+          <t>CV</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>P25</t>
+          <t>skewness</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>Median</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>P75</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>Max</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>P10</t>
-        </is>
-      </c>
-      <c r="K1" s="1" t="inlineStr">
-        <is>
-          <t>P33</t>
+          <t>slope_abs_mean</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>M</t>
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>PatientAge</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>665</v>
+        <v>1</v>
       </c>
       <c r="C2" t="n">
-        <v>149.52</v>
+        <v>0.113</v>
       </c>
       <c r="D2" t="n">
-        <v>27.46</v>
+        <v>0.08169999999999999</v>
       </c>
       <c r="E2" t="n">
-        <v>14</v>
+        <v>-0.2996</v>
       </c>
       <c r="F2" t="n">
-        <v>132</v>
+        <v>-0.2587</v>
       </c>
       <c r="G2" t="n">
-        <v>150</v>
-      </c>
-      <c r="H2" t="n">
-        <v>166</v>
-      </c>
-      <c r="I2" t="n">
-        <v>299</v>
-      </c>
-      <c r="J2" t="n">
-        <v>118</v>
-      </c>
-      <c r="K2" t="n">
-        <v>139</v>
+        <v>0.0795</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>F</t>
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>Sex</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>1008</v>
+        <v>0.113</v>
       </c>
       <c r="C3" t="n">
-        <v>104.69</v>
+        <v>1</v>
       </c>
       <c r="D3" t="n">
-        <v>15.71</v>
+        <v>0.1199</v>
       </c>
       <c r="E3" t="n">
-        <v>30</v>
+        <v>-0.3376</v>
       </c>
       <c r="F3" t="n">
-        <v>95</v>
+        <v>-0.3552</v>
       </c>
       <c r="G3" t="n">
-        <v>103</v>
-      </c>
-      <c r="H3" t="n">
-        <v>114</v>
-      </c>
-      <c r="I3" t="n">
-        <v>190</v>
-      </c>
-      <c r="J3" t="n">
-        <v>87</v>
-      </c>
-      <c r="K3" t="n">
-        <v>98</v>
+        <v>0.1567</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="1" t="inlineStr">
+        <is>
+          <t>mean</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>0.08169999999999999</v>
+      </c>
+      <c r="C4" t="n">
+        <v>0.1199</v>
+      </c>
+      <c r="D4" t="n">
+        <v>1</v>
+      </c>
+      <c r="E4" t="n">
+        <v>-0.2726</v>
+      </c>
+      <c r="F4" t="n">
+        <v>-0.376</v>
+      </c>
+      <c r="G4" t="n">
+        <v>0.4298</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="1" t="inlineStr">
+        <is>
+          <t>CV</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>-0.2996</v>
+      </c>
+      <c r="C5" t="n">
+        <v>-0.3376</v>
+      </c>
+      <c r="D5" t="n">
+        <v>-0.2726</v>
+      </c>
+      <c r="E5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F5" t="n">
+        <v>0.4456</v>
+      </c>
+      <c r="G5" t="n">
+        <v>0.1159</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="1" t="inlineStr">
+        <is>
+          <t>skewness</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>-0.2587</v>
+      </c>
+      <c r="C6" t="n">
+        <v>-0.3552</v>
+      </c>
+      <c r="D6" t="n">
+        <v>-0.376</v>
+      </c>
+      <c r="E6" t="n">
+        <v>0.4456</v>
+      </c>
+      <c r="F6" t="n">
+        <v>1</v>
+      </c>
+      <c r="G6" t="n">
+        <v>-0.1377</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="1" t="inlineStr">
+        <is>
+          <t>slope_abs_mean</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>0.0795</v>
+      </c>
+      <c r="C7" t="n">
+        <v>0.1567</v>
+      </c>
+      <c r="D7" t="n">
+        <v>0.4298</v>
+      </c>
+      <c r="E7" t="n">
+        <v>0.1159</v>
+      </c>
+      <c r="F7" t="n">
+        <v>-0.1377</v>
+      </c>
+      <c r="G7" t="n">
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -4369,13 +4346,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C32"/>
+  <dimension ref="A1:K3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Model</t>
+          <t>Sex</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
@@ -4385,411 +4362,122 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Pct</t>
+          <t>Mean</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>SD</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Min</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>P25</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Median</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>P75</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Max</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>P10</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>P33</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Sensation 64</t>
+          <t>M</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>585</v>
+        <v>665</v>
       </c>
       <c r="C2" t="n">
-        <v>35</v>
+        <v>149.52</v>
+      </c>
+      <c r="D2" t="n">
+        <v>27.46</v>
+      </c>
+      <c r="E2" t="n">
+        <v>14</v>
+      </c>
+      <c r="F2" t="n">
+        <v>132</v>
+      </c>
+      <c r="G2" t="n">
+        <v>150</v>
+      </c>
+      <c r="H2" t="n">
+        <v>166</v>
+      </c>
+      <c r="I2" t="n">
+        <v>299</v>
+      </c>
+      <c r="J2" t="n">
+        <v>118</v>
+      </c>
+      <c r="K2" t="n">
+        <v>139</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Revolution CT</t>
+          <t>F</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>382</v>
+        <v>1008</v>
       </c>
       <c r="C3" t="n">
-        <v>22.8</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>SOMATOM Definition AS+</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
-        <v>319</v>
-      </c>
-      <c r="C4" t="n">
-        <v>19.1</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Ingenuity Core 128</t>
-        </is>
-      </c>
-      <c r="B5" t="n">
-        <v>291</v>
-      </c>
-      <c r="C5" t="n">
-        <v>17.4</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>SOMATOM Definition Flash</t>
-        </is>
-      </c>
-      <c r="B6" t="n">
-        <v>15</v>
-      </c>
-      <c r="C6" t="n">
-        <v>0.9</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>LightSpeed VCT</t>
-        </is>
-      </c>
-      <c r="B7" t="n">
-        <v>8</v>
-      </c>
-      <c r="C7" t="n">
-        <v>0.5</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>SOMATOM Definition AS</t>
-        </is>
-      </c>
-      <c r="B8" t="n">
-        <v>7</v>
-      </c>
-      <c r="C8" t="n">
-        <v>0.4</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>iCT 256</t>
-        </is>
-      </c>
-      <c r="B9" t="n">
-        <v>7</v>
-      </c>
-      <c r="C9" t="n">
-        <v>0.4</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Aquilion</t>
-        </is>
-      </c>
-      <c r="B10" t="n">
-        <v>6</v>
-      </c>
-      <c r="C10" t="n">
-        <v>0.4</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>Brilliance 64</t>
-        </is>
-      </c>
-      <c r="B11" t="n">
-        <v>6</v>
-      </c>
-      <c r="C11" t="n">
-        <v>0.4</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>SOMATOM Definition Edge</t>
-        </is>
-      </c>
-      <c r="B12" t="n">
-        <v>6</v>
-      </c>
-      <c r="C12" t="n">
-        <v>0.4</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>Aquilion PRIME</t>
-        </is>
-      </c>
-      <c r="B13" t="n">
-        <v>5</v>
-      </c>
-      <c r="C13" t="n">
-        <v>0.3</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>Ingenuity CT</t>
-        </is>
-      </c>
-      <c r="B14" t="n">
-        <v>5</v>
-      </c>
-      <c r="C14" t="n">
-        <v>0.3</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>IQon - Spectral CT</t>
-        </is>
-      </c>
-      <c r="B15" t="n">
-        <v>3</v>
-      </c>
-      <c r="C15" t="n">
-        <v>0.2</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>SOMATOM Drive</t>
-        </is>
-      </c>
-      <c r="B16" t="n">
-        <v>3</v>
-      </c>
-      <c r="C16" t="n">
-        <v>0.2</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>Discovery CT750 HD</t>
-        </is>
-      </c>
-      <c r="B17" t="n">
-        <v>3</v>
-      </c>
-      <c r="C17" t="n">
-        <v>0.2</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>Emotion 6</t>
-        </is>
-      </c>
-      <c r="B18" t="n">
-        <v>3</v>
-      </c>
-      <c r="C18" t="n">
-        <v>0.2</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>SOMATOM Force</t>
-        </is>
-      </c>
-      <c r="B19" t="n">
-        <v>2</v>
-      </c>
-      <c r="C19" t="n">
-        <v>0.1</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>Optima CT660</t>
-        </is>
-      </c>
-      <c r="B20" t="n">
-        <v>2</v>
-      </c>
-      <c r="C20" t="n">
-        <v>0.1</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>SOMATOM Definition</t>
-        </is>
-      </c>
-      <c r="B21" t="n">
-        <v>2</v>
-      </c>
-      <c r="C21" t="n">
-        <v>0.1</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>Sensation 16</t>
-        </is>
-      </c>
-      <c r="B22" t="n">
-        <v>2</v>
-      </c>
-      <c r="C22" t="n">
-        <v>0.1</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>Brivo CT385 Series</t>
-        </is>
-      </c>
-      <c r="B23" t="n">
-        <v>2</v>
-      </c>
-      <c r="C23" t="n">
-        <v>0.1</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>Aquilion ONE</t>
-        </is>
-      </c>
-      <c r="B24" t="n">
-        <v>1</v>
-      </c>
-      <c r="C24" t="n">
-        <v>0.1</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>Emotion 16</t>
-        </is>
-      </c>
-      <c r="B25" t="n">
-        <v>1</v>
-      </c>
-      <c r="C25" t="n">
-        <v>0.1</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>iCT 128</t>
-        </is>
-      </c>
-      <c r="B26" t="n">
-        <v>1</v>
-      </c>
-      <c r="C26" t="n">
-        <v>0.1</v>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>Scope</t>
-        </is>
-      </c>
-      <c r="B27" t="n">
-        <v>1</v>
-      </c>
-      <c r="C27" t="n">
-        <v>0.1</v>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>BrightSpeed</t>
-        </is>
-      </c>
-      <c r="B28" t="n">
-        <v>1</v>
-      </c>
-      <c r="C28" t="n">
-        <v>0.1</v>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>LightSpeed16</t>
-        </is>
-      </c>
-      <c r="B29" t="n">
-        <v>1</v>
-      </c>
-      <c r="C29" t="n">
-        <v>0.1</v>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>Revolution EVO</t>
-        </is>
-      </c>
-      <c r="B30" t="n">
-        <v>1</v>
-      </c>
-      <c r="C30" t="n">
-        <v>0.1</v>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>BrightSpeed S</t>
-        </is>
-      </c>
-      <c r="B31" t="n">
-        <v>1</v>
-      </c>
-      <c r="C31" t="n">
-        <v>0.1</v>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>SOMATOM Perspective</t>
-        </is>
-      </c>
-      <c r="B32" t="n">
-        <v>1</v>
-      </c>
-      <c r="C32" t="n">
-        <v>0.1</v>
+        <v>104.69</v>
+      </c>
+      <c r="D3" t="n">
+        <v>15.71</v>
+      </c>
+      <c r="E3" t="n">
+        <v>30</v>
+      </c>
+      <c r="F3" t="n">
+        <v>95</v>
+      </c>
+      <c r="G3" t="n">
+        <v>103</v>
+      </c>
+      <c r="H3" t="n">
+        <v>114</v>
+      </c>
+      <c r="I3" t="n">
+        <v>190</v>
+      </c>
+      <c r="J3" t="n">
+        <v>87</v>
+      </c>
+      <c r="K3" t="n">
+        <v>98</v>
       </c>
     </row>
   </sheetData>
@@ -4803,6 +4491,440 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:C32"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Model</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Pct</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Sensation 64</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>585</v>
+      </c>
+      <c r="C2" t="n">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Revolution CT</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>382</v>
+      </c>
+      <c r="C3" t="n">
+        <v>22.8</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>SOMATOM Definition AS+</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>319</v>
+      </c>
+      <c r="C4" t="n">
+        <v>19.1</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Ingenuity Core 128</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>291</v>
+      </c>
+      <c r="C5" t="n">
+        <v>17.4</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>SOMATOM Definition Flash</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>15</v>
+      </c>
+      <c r="C6" t="n">
+        <v>0.9</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>LightSpeed VCT</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>8</v>
+      </c>
+      <c r="C7" t="n">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>SOMATOM Definition AS</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>7</v>
+      </c>
+      <c r="C8" t="n">
+        <v>0.4</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>iCT 256</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>7</v>
+      </c>
+      <c r="C9" t="n">
+        <v>0.4</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Aquilion</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>6</v>
+      </c>
+      <c r="C10" t="n">
+        <v>0.4</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Brilliance 64</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>6</v>
+      </c>
+      <c r="C11" t="n">
+        <v>0.4</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>SOMATOM Definition Edge</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>6</v>
+      </c>
+      <c r="C12" t="n">
+        <v>0.4</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Aquilion PRIME</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>5</v>
+      </c>
+      <c r="C13" t="n">
+        <v>0.3</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Ingenuity CT</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>5</v>
+      </c>
+      <c r="C14" t="n">
+        <v>0.3</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>IQon - Spectral CT</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>3</v>
+      </c>
+      <c r="C15" t="n">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>SOMATOM Drive</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>3</v>
+      </c>
+      <c r="C16" t="n">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Discovery CT750 HD</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>3</v>
+      </c>
+      <c r="C17" t="n">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Emotion 6</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>3</v>
+      </c>
+      <c r="C18" t="n">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>SOMATOM Force</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>2</v>
+      </c>
+      <c r="C19" t="n">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Optima CT660</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>2</v>
+      </c>
+      <c r="C20" t="n">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>SOMATOM Definition</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>2</v>
+      </c>
+      <c r="C21" t="n">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Sensation 16</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>2</v>
+      </c>
+      <c r="C22" t="n">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Brivo CT385 Series</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>2</v>
+      </c>
+      <c r="C23" t="n">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Aquilion ONE</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>1</v>
+      </c>
+      <c r="C24" t="n">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Emotion 16</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>1</v>
+      </c>
+      <c r="C25" t="n">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>iCT 128</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>1</v>
+      </c>
+      <c r="C26" t="n">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Scope</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>1</v>
+      </c>
+      <c r="C27" t="n">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>BrightSpeed</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>1</v>
+      </c>
+      <c r="C28" t="n">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>LightSpeed16</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>1</v>
+      </c>
+      <c r="C29" t="n">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Revolution EVO</t>
+        </is>
+      </c>
+      <c r="B30" t="n">
+        <v>1</v>
+      </c>
+      <c r="C30" t="n">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>BrightSpeed S</t>
+        </is>
+      </c>
+      <c r="B31" t="n">
+        <v>1</v>
+      </c>
+      <c r="C31" t="n">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>SOMATOM Perspective</t>
+        </is>
+      </c>
+      <c r="B32" t="n">
+        <v>1</v>
+      </c>
+      <c r="C32" t="n">
+        <v>0.1</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:C8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>

</xml_diff>